<commit_message>
Update third shift route and bus schedule
</commit_message>
<xml_diff>
--- a/employees.xlsx
+++ b/employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BHARTESH\OneDrive\Desktop\updated project\SHARED SUPPORT SERVICE APP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641E5CEF-CCED-4FA0-8D34-8BD5974EB7DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E72A63-85C0-43C3-A211-13F7364D767B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9060" uniqueCount="2466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9059" uniqueCount="2466">
   <si>
     <t>employeeCode</t>
   </si>
@@ -55632,7 +55632,7 @@
         <v>9938097309</v>
       </c>
       <c r="D1412" s="3" t="s">
-        <v>1746</v>
+        <v>1807</v>
       </c>
       <c r="E1412" s="5" t="str">
         <f t="shared" ref="E1412:E1475" si="22">LOWER(SUBSTITUTE(B1412," ",""))&amp;"@gmail.com"</f>
@@ -55642,17 +55642,17 @@
         <v>15</v>
       </c>
       <c r="G1412" s="4" t="s">
-        <v>1169</v>
+        <v>1245</v>
       </c>
       <c r="H1412" s="6">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="I1412" s="6"/>
       <c r="J1412" s="2">
         <v>229085</v>
       </c>
-      <c r="K1412" s="4" t="s">
-        <v>433</v>
+      <c r="K1412" s="4">
+        <v>22</v>
       </c>
     </row>
     <row r="1413" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>